<commit_message>
Matriz de rastreabilidade atualizada
</commit_message>
<xml_diff>
--- a/Matriz de rastreabilidade Tech Music.xlsx
+++ b/Matriz de rastreabilidade Tech Music.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="502" documentId="11_92485C45C1F39E42E268565A893E8C18510380CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF6A723E-ACEB-4DCB-ABA0-D6F15C423AB2}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell\Downloads\documentary-repository\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7CC7E5C-C88D-48BE-A721-D3F42A9EB2CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -23,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -650,7 +653,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -749,12 +752,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -772,6 +769,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -812,7 +815,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1109,19 +1112,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:K26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="38.28515625" customWidth="1"/>
-    <col min="5" max="5" width="14.140625" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.109375" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="36.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:11">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -1153,7 +1156,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:11" ht="60.75">
+    <row r="4" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B4" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF01</v>
@@ -1186,7 +1189,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="60.75">
+    <row r="5" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B5" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF02</v>
@@ -1219,7 +1222,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="76.5">
+    <row r="6" spans="2:11" ht="72" x14ac:dyDescent="0.3">
       <c r="B6" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF03</v>
@@ -1252,7 +1255,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="76.5">
+    <row r="7" spans="2:11" ht="72" x14ac:dyDescent="0.3">
       <c r="B7" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF04</v>
@@ -1276,7 +1279,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="60.75">
+    <row r="8" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B8" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF05</v>
@@ -1300,7 +1303,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="60.75">
+    <row r="9" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B9" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF06</v>
@@ -1318,7 +1321,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="45.75">
+    <row r="10" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B10" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF07</v>
@@ -1333,7 +1336,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="45.75">
+    <row r="11" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B11" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF08</v>
@@ -1348,7 +1351,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="2:11" ht="60.75">
+    <row r="12" spans="2:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B12" t="str">
         <f>"RF0" &amp; TEXT(ROW() - ROW(Tabela1[[#Headers],[ID]]), "0;-0")</f>
         <v>RF09</v>
@@ -1363,7 +1366,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="2:11" ht="30.75">
+    <row r="13" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>51</v>
       </c>
@@ -1377,7 +1380,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:11" ht="45.75">
+    <row r="14" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>55</v>
       </c>
@@ -1391,7 +1394,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="2:11" ht="45.75">
+    <row r="15" spans="2:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>59</v>
       </c>
@@ -1405,7 +1408,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="2:11" ht="30.75">
+    <row r="16" spans="2:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>63</v>
       </c>
@@ -1419,7 +1422,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="2:10">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>67</v>
       </c>
@@ -1448,7 +1451,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="2:10">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>72</v>
       </c>
@@ -1477,7 +1480,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="2:10">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>51</v>
       </c>
@@ -1503,7 +1506,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="30.75">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>55</v>
       </c>
@@ -1529,7 +1532,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="26" spans="2:10" ht="30.75">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>59</v>
       </c>
@@ -1566,840 +1569,840 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{137BDAF4-8877-4BBC-B957-C26603140F9C}">
   <dimension ref="B1:J29"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10">
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B1" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-    </row>
-    <row r="2" spans="2:10">
-      <c r="B2" s="4" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+    </row>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="7" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="45.75">
-      <c r="B3" s="5" t="s">
+    <row r="3" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B3" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="8" t="s">
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I4" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" ht="30.75">
-      <c r="B4" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="8" t="s">
+      <c r="J4" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B8" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B10" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="5" t="s">
+      <c r="H10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J10" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="30.75">
-      <c r="B5" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="8" t="s">
+    <row r="11" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B11" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="5" t="s">
+      <c r="H11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I11" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J11" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B12" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B13" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B14" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B15" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B16" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B17" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B18" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B19" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B23" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B24" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="30.75">
-      <c r="B6" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="8" t="s">
+    <row r="25" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G26" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B27" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G27" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" ht="30.75">
-      <c r="B7" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" ht="30.75">
-      <c r="B8" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="8" t="s">
+      <c r="H27" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B28" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.3">
+      <c r="B29" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" ht="30.75">
-      <c r="B9" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" ht="30.75">
-      <c r="B10" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="11" spans="2:10" ht="30.75">
-      <c r="B11" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" ht="30.75">
-      <c r="B12" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="I12" s="6" t="s">
+      <c r="G29" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="I29" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="J12" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" ht="30.75">
-      <c r="B13" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" ht="30.75">
-      <c r="B14" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I14" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="15" spans="2:10" ht="30.75">
-      <c r="B15" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="16" spans="2:10" ht="30.75">
-      <c r="B16" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" ht="30.75">
-      <c r="B17" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" ht="30.75">
-      <c r="B18" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H18" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J18" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" ht="30.75">
-      <c r="B19" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" ht="30.75">
-      <c r="B20" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J20" s="5" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="21" spans="2:10" ht="20.25" customHeight="1">
-      <c r="B21" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="22" spans="2:10" ht="30.75">
-      <c r="B22" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="I22" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="J22" s="5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="23" spans="2:10" ht="30.75">
-      <c r="B23" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="J23" s="5" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="24" spans="2:10" ht="30.75">
-      <c r="B24" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F24" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="J24" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="25" spans="2:10" ht="30.75">
-      <c r="B25" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="26" spans="2:10" ht="30.75">
-      <c r="B26" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="J26" s="5" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="27" spans="2:10" ht="30.75">
-      <c r="B27" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="J27" s="5" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="28" spans="2:10" ht="30.75">
-      <c r="B28" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>136</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="I28" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="J28" s="5" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="29" spans="2:10" ht="30.75">
-      <c r="B29" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="F29" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="J29" s="5" t="s">
+      <c r="J29" s="3" t="s">
         <v>203</v>
       </c>
     </row>

</xml_diff>